<commit_message>
Fixed the length issue of the cross system mode
</commit_message>
<xml_diff>
--- a/backend/outputs/CrossSystem_Winner_Output.xlsx
+++ b/backend/outputs/CrossSystem_Winner_Output.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -581,8 +581,10 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>70116</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -656,7 +658,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -669,8 +671,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>70611</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>70611</t>
+        </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -744,7 +748,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>BRIDGEPORT</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -757,8 +761,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>8014</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -832,7 +838,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ANCHORAGE</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -845,8 +851,10 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>99501</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>99501</t>
+        </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -920,7 +928,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>HAMILTON</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -933,8 +941,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>45011</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>45011</t>
+        </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1008,7 +1018,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>ASHLAND</t>
+          <t>Ashland</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1021,8 +1031,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>44805</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>44805</t>
+        </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1096,7 +1108,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CHICAGO</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1109,8 +1121,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>60632</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>60632</t>
+        </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1184,7 +1198,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1197,8 +1211,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>95111</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1272,7 +1288,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SAN JOS</t>
+          <t>San Jos</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1285,8 +1301,10 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>95111</v>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1360,7 +1378,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1373,8 +1391,10 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>21224</v>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1448,7 +1468,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1461,8 +1481,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>21224</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1536,7 +1558,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MIDDLE ISLAND</t>
+          <t>Middle Island</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1549,8 +1571,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>11953</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>11953</t>
+        </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1624,7 +1648,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>LOS ANGELES</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1637,8 +1661,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>90034</v>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>90034</t>
+        </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1712,7 +1738,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CHAGRIN FALLS</t>
+          <t>Chagrin Falls</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1725,8 +1751,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>44023</v>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>44023</t>
+        </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1800,7 +1828,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>LAREDO</t>
+          <t>Laredo</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1813,8 +1841,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>78045</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>78045</t>
+        </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1888,7 +1918,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>PHOENIX</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1901,8 +1931,10 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>85013</v>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>85013</t>
+        </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1976,7 +2008,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MC MINNVILLE</t>
+          <t>Mc Minnville</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1989,8 +2021,10 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>37110</v>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>37110</t>
+        </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2064,7 +2098,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MILWAUKEE</t>
+          <t>Milwaukee</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2077,8 +2111,10 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>53207</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>53207</t>
+        </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -2152,7 +2188,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TAYLOR</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2165,8 +2201,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>48180</v>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>48180</t>
+        </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2240,7 +2278,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ROCKFORD</t>
+          <t>Rockford</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2253,8 +2291,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>61109</v>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>61109</t>
+        </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2328,7 +2368,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ASTON</t>
+          <t>Aston</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2341,8 +2381,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>19014</v>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>19014</t>
+        </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2416,7 +2458,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2429,8 +2471,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>95111</v>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2504,7 +2548,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>IRVING</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2517,8 +2561,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>75062</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>75062</t>
+        </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2592,7 +2638,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ALBANY</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2605,8 +2651,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>12204</v>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>12204</t>
+        </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2680,7 +2728,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2693,8 +2741,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>8846</v>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2768,7 +2818,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2781,8 +2831,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>8846</v>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2856,7 +2908,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2869,8 +2921,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>8846</v>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2944,7 +2998,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2957,8 +3011,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>8846</v>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -3032,7 +3088,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3045,8 +3101,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>8846</v>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -3236,7 +3294,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -3249,8 +3307,10 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>70116</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -3324,7 +3384,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -3337,8 +3397,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>70611</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>70611</t>
+        </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -3412,7 +3474,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>BRIDGEPORT</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -3425,8 +3487,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>8014</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -3500,7 +3564,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ANCHORAGE</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -3513,8 +3577,10 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>99501</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>99501</t>
+        </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -3588,7 +3654,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>HAMILTON</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3601,8 +3667,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>45011</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>45011</t>
+        </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3676,7 +3744,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>ASHLAND</t>
+          <t>Ashland</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -3689,8 +3757,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>44805</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>44805</t>
+        </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3764,7 +3834,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CHICAGO</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3777,8 +3847,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>60632</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>60632</t>
+        </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -3852,7 +3924,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3865,8 +3937,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>95111</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -3940,7 +4014,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SAN JOS</t>
+          <t>San Jos</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3953,8 +4027,10 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>95111</v>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -4028,7 +4104,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -4041,8 +4117,10 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>21224</v>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -4116,7 +4194,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4129,8 +4207,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>21224</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -4204,7 +4284,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MIDDLE ISLAND</t>
+          <t>Middle Island</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -4217,8 +4297,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>11953</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>11953</t>
+        </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -4292,7 +4374,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>LOS ANGELES</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -4305,8 +4387,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>90034</v>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>90034</t>
+        </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -4380,7 +4464,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CHAGRIN FALLS</t>
+          <t>Chagrin Falls</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -4393,8 +4477,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>44023</v>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>44023</t>
+        </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -4468,7 +4554,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>LAREDO</t>
+          <t>Laredo</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -4481,8 +4567,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>78045</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>78045</t>
+        </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -4556,7 +4644,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>PHOENIX</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -4569,8 +4657,10 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>85013</v>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>85013</t>
+        </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -4644,7 +4734,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MC MINNVILLE</t>
+          <t>Mc Minnville</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -4657,8 +4747,10 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>37110</v>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>37110</t>
+        </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -4732,7 +4824,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MILWAUKEE</t>
+          <t>Milwaukee</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -4745,8 +4837,10 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>53207</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>53207</t>
+        </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -4820,7 +4914,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TAYLOR</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -4833,8 +4927,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>48180</v>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>48180</t>
+        </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -4908,7 +5004,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ROCKFORD</t>
+          <t>Rockford</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -4921,8 +5017,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>61109</v>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>61109</t>
+        </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -4996,7 +5094,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ASTON</t>
+          <t>Aston</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -5009,8 +5107,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>19014</v>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>19014</t>
+        </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -5084,7 +5184,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -5097,8 +5197,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>95111</v>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -5172,7 +5274,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>IRVING</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -5185,8 +5287,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>75062</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>75062</t>
+        </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -5260,7 +5364,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ALBANY</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -5273,8 +5377,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>12204</v>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>12204</t>
+        </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -5348,7 +5454,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -5361,8 +5467,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>8846</v>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -5436,7 +5544,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -5449,8 +5557,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>8846</v>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -5524,7 +5634,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -5537,8 +5647,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>8846</v>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -5612,7 +5724,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -5625,8 +5737,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>8846</v>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -5700,7 +5814,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -5713,8 +5827,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>8846</v>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -5904,7 +6020,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -5917,8 +6033,10 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>70116</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -5992,7 +6110,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -6005,8 +6123,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>70611</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>70611</t>
+        </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -6080,7 +6200,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>BRIDGEPORT</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -6093,8 +6213,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>8014</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -6168,7 +6290,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ANCHORAGE</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -6181,8 +6303,10 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>99501</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>99501</t>
+        </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -6256,7 +6380,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>HAMILTON</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -6269,8 +6393,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>45011</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>45011</t>
+        </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -6344,7 +6470,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>ASHLAND</t>
+          <t>Ashland</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -6357,8 +6483,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>44805</v>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>44805</t>
+        </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -6432,7 +6560,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CHICAGO</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -6445,8 +6573,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>60632</v>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>60632</t>
+        </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -6520,7 +6650,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -6533,8 +6663,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>95111</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -6608,7 +6740,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SAN JOS</t>
+          <t>San Jos</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -6621,8 +6753,10 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>95111</v>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -6696,7 +6830,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -6709,8 +6843,10 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>21224</v>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -6784,7 +6920,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -6797,8 +6933,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>21224</v>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -6872,7 +7010,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MIDDLE ISLAND</t>
+          <t>Middle Island</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -6885,8 +7023,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>11953</v>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>11953</t>
+        </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -6960,7 +7100,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>LOS ANGELES</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -6973,8 +7113,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>90034</v>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>90034</t>
+        </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -7048,7 +7190,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CHAGRIN FALLS</t>
+          <t>Chagrin Falls</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -7061,8 +7203,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>44023</v>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>44023</t>
+        </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -7136,7 +7280,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>LAREDO</t>
+          <t>Laredo</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -7149,8 +7293,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>78045</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>78045</t>
+        </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -7224,7 +7370,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>PHOENIX</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -7237,8 +7383,10 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>85013</v>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>85013</t>
+        </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -7312,7 +7460,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MC MINNVILLE</t>
+          <t>Mc Minnville</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -7325,8 +7473,10 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>37110</v>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>37110</t>
+        </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -7400,7 +7550,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MILWAUKEE</t>
+          <t>Milwaukee</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -7413,8 +7563,10 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>53207</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>53207</t>
+        </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -7488,7 +7640,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TAYLOR</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -7501,8 +7653,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>48180</v>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>48180</t>
+        </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -7576,7 +7730,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ROCKFORD</t>
+          <t>Rockford</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -7589,8 +7743,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>61109</v>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>61109</t>
+        </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -7664,7 +7820,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ASTON</t>
+          <t>Aston</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -7677,8 +7833,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>19014</v>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>19014</t>
+        </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -7752,7 +7910,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -7765,8 +7923,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>95111</v>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -7840,7 +8000,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>IRVING</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -7853,8 +8013,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>75062</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>75062</t>
+        </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -7928,7 +8090,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ALBANY</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -7941,8 +8103,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>12204</v>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>12204</t>
+        </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -8016,7 +8180,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -8029,8 +8193,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>8846</v>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -8104,7 +8270,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -8117,8 +8283,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>8846</v>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -8192,7 +8360,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -8205,8 +8373,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>8846</v>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -8280,7 +8450,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -8293,8 +8463,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>8846</v>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -8368,7 +8540,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -8381,8 +8553,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>8846</v>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -8456,7 +8630,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -8469,8 +8643,10 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>70116</v>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -8544,7 +8720,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -8557,8 +8733,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>70611</v>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>70611</t>
+        </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -8632,7 +8810,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>BRIDGEPORT</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -8645,8 +8823,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>8014</v>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -8720,7 +8900,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ANCHORAGE</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -8733,8 +8913,10 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>99501</v>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>99501</t>
+        </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -8808,7 +8990,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>HAMILTON</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -8821,8 +9003,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>45011</v>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>45011</t>
+        </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -8896,7 +9080,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>ASHLAND</t>
+          <t>Ashland</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -8909,8 +9093,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>44805</v>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>44805</t>
+        </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -8984,7 +9170,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>CHICAGO</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -8997,8 +9183,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>60632</v>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>60632</t>
+        </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -9072,7 +9260,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -9085,8 +9273,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>95111</v>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -9160,7 +9350,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>SAN JOS</t>
+          <t>San Jos</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -9173,8 +9363,10 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>95111</v>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -9248,7 +9440,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -9261,8 +9453,10 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>21224</v>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -9336,7 +9530,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -9349,8 +9543,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>21224</v>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -9424,7 +9620,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>MIDDLE ISLAND</t>
+          <t>Middle Island</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -9437,8 +9633,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>11953</v>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>11953</t>
+        </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -9512,7 +9710,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>LOS ANGELES</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -9525,8 +9723,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>90034</v>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>90034</t>
+        </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -9600,7 +9800,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>CHAGRIN FALLS</t>
+          <t>Chagrin Falls</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -9613,8 +9813,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>44023</v>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>44023</t>
+        </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -9688,7 +9890,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>LAREDO</t>
+          <t>Laredo</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -9701,8 +9903,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>78045</v>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>78045</t>
+        </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -9776,7 +9980,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>PHOENIX</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -9789,8 +9993,10 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>85013</v>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>85013</t>
+        </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -9864,7 +10070,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>MC MINNVILLE</t>
+          <t>Mc Minnville</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -9877,8 +10083,10 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>37110</v>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>37110</t>
+        </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -9952,7 +10160,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>MILWAUKEE</t>
+          <t>Milwaukee</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -9965,8 +10173,10 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>53207</v>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>53207</t>
+        </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -10040,7 +10250,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>TAYLOR</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -10053,8 +10263,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>48180</v>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>48180</t>
+        </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -10128,7 +10340,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>ROCKFORD</t>
+          <t>Rockford</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -10141,8 +10353,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J50" t="n">
-        <v>61109</v>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>61109</t>
+        </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -10216,7 +10430,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>ASTON</t>
+          <t>Aston</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -10229,8 +10443,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>19014</v>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>19014</t>
+        </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -10304,7 +10520,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -10317,8 +10533,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J52" t="n">
-        <v>95111</v>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -10392,7 +10610,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>IRVING</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -10405,8 +10623,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J53" t="n">
-        <v>75062</v>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>75062</t>
+        </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -10480,7 +10700,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>ALBANY</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -10493,8 +10713,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>12204</v>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>12204</t>
+        </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -10568,7 +10790,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -10581,8 +10803,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>8846</v>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -10656,7 +10880,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -10669,8 +10893,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J56" t="n">
-        <v>8846</v>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -10744,7 +10970,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -10757,8 +10983,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>8846</v>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -10832,7 +11060,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -10845,8 +11073,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>8846</v>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -10920,7 +11150,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -10933,8 +11163,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J59" t="n">
-        <v>8846</v>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -11008,7 +11240,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -11021,8 +11253,10 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J60" t="n">
-        <v>70116</v>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>70116</t>
+        </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -11096,7 +11330,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>NEW ORLEANS</t>
+          <t>New Orleans</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -11109,8 +11343,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J61" t="n">
-        <v>70611</v>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>70611</t>
+        </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -11184,7 +11420,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>BRIDGEPORT</t>
+          <t>Bridgeport</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -11197,8 +11433,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J62" t="n">
-        <v>8014</v>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -11272,7 +11510,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>ANCHORAGE</t>
+          <t>Anchorage</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -11285,8 +11523,10 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J63" t="n">
-        <v>99501</v>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>99501</t>
+        </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -11360,7 +11600,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>HAMILTON</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -11373,8 +11613,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J64" t="n">
-        <v>45011</v>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>45011</t>
+        </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -11448,7 +11690,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>ASHLAND</t>
+          <t>Ashland</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -11461,8 +11703,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J65" t="n">
-        <v>44805</v>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>44805</t>
+        </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -11536,7 +11780,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>CHICAGO</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -11549,8 +11793,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J66" t="n">
-        <v>60632</v>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>60632</t>
+        </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -11624,7 +11870,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -11637,8 +11883,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J67" t="n">
-        <v>95111</v>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -11712,7 +11960,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>SAN JOS</t>
+          <t>San Jos</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -11725,8 +11973,10 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J68" t="n">
-        <v>95111</v>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -11800,7 +12050,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -11813,8 +12063,10 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J69" t="n">
-        <v>21224</v>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -11888,7 +12140,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>BALTIMORE</t>
+          <t>Baltimore</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -11901,8 +12153,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J70" t="n">
-        <v>21224</v>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>21224</t>
+        </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -11976,7 +12230,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>MIDDLE ISLAND</t>
+          <t>Middle Island</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -11989,8 +12243,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J71" t="n">
-        <v>11953</v>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>11953</t>
+        </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -12064,7 +12320,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>LOS ANGELES</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -12077,8 +12333,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J72" t="n">
-        <v>90034</v>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>90034</t>
+        </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -12152,7 +12410,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>CHAGRIN FALLS</t>
+          <t>Chagrin Falls</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -12165,8 +12423,10 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J73" t="n">
-        <v>44023</v>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>44023</t>
+        </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -12240,7 +12500,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>LAREDO</t>
+          <t>Laredo</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -12253,8 +12513,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J74" t="n">
-        <v>78045</v>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>78045</t>
+        </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -12328,7 +12590,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>PHOENIX</t>
+          <t>Phoenix</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -12341,8 +12603,10 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J75" t="n">
-        <v>85013</v>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>85013</t>
+        </is>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -12416,7 +12680,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>MC MINNVILLE</t>
+          <t>Mc Minnville</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -12429,8 +12693,10 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J76" t="n">
-        <v>37110</v>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>37110</t>
+        </is>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -12504,7 +12770,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>MILWAUKEE</t>
+          <t>Milwaukee</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -12517,8 +12783,10 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J77" t="n">
-        <v>53207</v>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>53207</t>
+        </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -12592,7 +12860,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>TAYLOR</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -12605,8 +12873,10 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J78" t="n">
-        <v>48180</v>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>48180</t>
+        </is>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -12680,7 +12950,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>ROCKFORD</t>
+          <t>Rockford</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -12693,8 +12963,10 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J79" t="n">
-        <v>61109</v>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>61109</t>
+        </is>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -12768,7 +13040,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>ASTON</t>
+          <t>Aston</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -12781,8 +13053,10 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J80" t="n">
-        <v>19014</v>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>19014</t>
+        </is>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -12856,7 +13130,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>SAN JOSE</t>
+          <t>San Jose</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -12869,8 +13143,10 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J81" t="n">
-        <v>95111</v>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>95111</t>
+        </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -12944,7 +13220,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>IRVING</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -12957,8 +13233,10 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J82" t="n">
-        <v>75062</v>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>75062</t>
+        </is>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -13032,7 +13310,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>ALBANY</t>
+          <t>Albany</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -13045,8 +13323,10 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J83" t="n">
-        <v>12204</v>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>12204</t>
+        </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -13120,7 +13400,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -13133,8 +13413,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J84" t="n">
-        <v>8846</v>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -13208,7 +13490,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -13221,8 +13503,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J85" t="n">
-        <v>8846</v>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -13296,7 +13580,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -13309,8 +13593,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J86" t="n">
-        <v>8846</v>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -13384,7 +13670,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -13397,8 +13683,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J87" t="n">
-        <v>8846</v>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -13472,7 +13760,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>MIDDLESEX</t>
+          <t>Middlesex</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -13485,8 +13773,10 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J88" t="n">
-        <v>8846</v>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>8846</t>
+        </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fixed the  ui issue till the processing part
</commit_message>
<xml_diff>
--- a/backend/outputs/CrossSystem_Winner_Output.xlsx
+++ b/backend/outputs/CrossSystem_Winner_Output.xlsx
@@ -581,10 +581,8 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>70116</t>
-        </is>
+      <c r="J2" t="n">
+        <v>70116</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -671,10 +669,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>70611</t>
-        </is>
+      <c r="J3" t="n">
+        <v>70611</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -761,10 +757,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>8014</t>
-        </is>
+      <c r="J4" t="n">
+        <v>8014</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -851,10 +845,8 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>99501</t>
-        </is>
+      <c r="J5" t="n">
+        <v>99501</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -941,10 +933,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>45011</t>
-        </is>
+      <c r="J6" t="n">
+        <v>45011</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1031,10 +1021,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>44805</t>
-        </is>
+      <c r="J7" t="n">
+        <v>44805</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1121,10 +1109,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>60632</t>
-        </is>
+      <c r="J8" t="n">
+        <v>60632</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1211,10 +1197,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J9" t="n">
+        <v>95111</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1301,10 +1285,8 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J10" t="n">
+        <v>95111</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1391,10 +1373,8 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J11" t="n">
+        <v>21224</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1481,10 +1461,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J12" t="n">
+        <v>21224</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1571,10 +1549,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>11953</t>
-        </is>
+      <c r="J13" t="n">
+        <v>11953</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1661,10 +1637,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>90034</t>
-        </is>
+      <c r="J14" t="n">
+        <v>90034</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1751,10 +1725,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>44023</t>
-        </is>
+      <c r="J15" t="n">
+        <v>44023</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1841,10 +1813,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>78045</t>
-        </is>
+      <c r="J16" t="n">
+        <v>78045</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1931,10 +1901,8 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>85013</t>
-        </is>
+      <c r="J17" t="n">
+        <v>85013</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2021,10 +1989,8 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>37110</t>
-        </is>
+      <c r="J18" t="n">
+        <v>37110</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2111,10 +2077,8 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>53207</t>
-        </is>
+      <c r="J19" t="n">
+        <v>53207</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -2201,10 +2165,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>48180</t>
-        </is>
+      <c r="J20" t="n">
+        <v>48180</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2291,10 +2253,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>61109</t>
-        </is>
+      <c r="J21" t="n">
+        <v>61109</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2381,10 +2341,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>19014</t>
-        </is>
+      <c r="J22" t="n">
+        <v>19014</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2471,10 +2429,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J23" t="n">
+        <v>95111</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2561,10 +2517,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>75062</t>
-        </is>
+      <c r="J24" t="n">
+        <v>75062</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2651,10 +2605,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>12204</t>
-        </is>
+      <c r="J25" t="n">
+        <v>12204</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2741,10 +2693,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J26" t="n">
+        <v>8846</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2831,10 +2781,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J27" t="n">
+        <v>8846</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2921,10 +2869,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J28" t="n">
+        <v>8846</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -3011,10 +2957,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J29" t="n">
+        <v>8846</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -3101,10 +3045,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J30" t="n">
+        <v>8846</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -3307,10 +3249,8 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>70116</t>
-        </is>
+      <c r="J2" t="n">
+        <v>70116</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -3397,10 +3337,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>70611</t>
-        </is>
+      <c r="J3" t="n">
+        <v>70611</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -3487,10 +3425,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>8014</t>
-        </is>
+      <c r="J4" t="n">
+        <v>8014</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -3577,10 +3513,8 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>99501</t>
-        </is>
+      <c r="J5" t="n">
+        <v>99501</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -3667,10 +3601,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>45011</t>
-        </is>
+      <c r="J6" t="n">
+        <v>45011</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -3757,10 +3689,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>44805</t>
-        </is>
+      <c r="J7" t="n">
+        <v>44805</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3847,10 +3777,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>60632</t>
-        </is>
+      <c r="J8" t="n">
+        <v>60632</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -3937,10 +3865,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J9" t="n">
+        <v>95111</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -4027,10 +3953,8 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J10" t="n">
+        <v>95111</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -4117,10 +4041,8 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J11" t="n">
+        <v>21224</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -4207,10 +4129,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J12" t="n">
+        <v>21224</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -4297,10 +4217,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>11953</t>
-        </is>
+      <c r="J13" t="n">
+        <v>11953</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -4387,10 +4305,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>90034</t>
-        </is>
+      <c r="J14" t="n">
+        <v>90034</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -4477,10 +4393,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>44023</t>
-        </is>
+      <c r="J15" t="n">
+        <v>44023</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -4567,10 +4481,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>78045</t>
-        </is>
+      <c r="J16" t="n">
+        <v>78045</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -4657,10 +4569,8 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>85013</t>
-        </is>
+      <c r="J17" t="n">
+        <v>85013</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -4747,10 +4657,8 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>37110</t>
-        </is>
+      <c r="J18" t="n">
+        <v>37110</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -4837,10 +4745,8 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>53207</t>
-        </is>
+      <c r="J19" t="n">
+        <v>53207</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -4927,10 +4833,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>48180</t>
-        </is>
+      <c r="J20" t="n">
+        <v>48180</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -5017,10 +4921,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>61109</t>
-        </is>
+      <c r="J21" t="n">
+        <v>61109</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -5107,10 +5009,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>19014</t>
-        </is>
+      <c r="J22" t="n">
+        <v>19014</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -5197,10 +5097,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J23" t="n">
+        <v>95111</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -5287,10 +5185,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>75062</t>
-        </is>
+      <c r="J24" t="n">
+        <v>75062</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -5377,10 +5273,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>12204</t>
-        </is>
+      <c r="J25" t="n">
+        <v>12204</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -5467,10 +5361,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J26" t="n">
+        <v>8846</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -5557,10 +5449,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J27" t="n">
+        <v>8846</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -5647,10 +5537,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J28" t="n">
+        <v>8846</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -5737,10 +5625,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J29" t="n">
+        <v>8846</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -5827,10 +5713,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J30" t="n">
+        <v>8846</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -6033,10 +5917,8 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>70116</t>
-        </is>
+      <c r="J2" t="n">
+        <v>70116</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -6123,10 +6005,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>70611</t>
-        </is>
+      <c r="J3" t="n">
+        <v>70611</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -6213,10 +6093,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>8014</t>
-        </is>
+      <c r="J4" t="n">
+        <v>8014</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -6303,10 +6181,8 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>99501</t>
-        </is>
+      <c r="J5" t="n">
+        <v>99501</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -6393,10 +6269,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>45011</t>
-        </is>
+      <c r="J6" t="n">
+        <v>45011</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -6483,10 +6357,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>44805</t>
-        </is>
+      <c r="J7" t="n">
+        <v>44805</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -6573,10 +6445,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>60632</t>
-        </is>
+      <c r="J8" t="n">
+        <v>60632</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -6663,10 +6533,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J9" t="n">
+        <v>95111</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -6753,10 +6621,8 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J10" t="n">
+        <v>95111</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -6843,10 +6709,8 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J11" t="n">
+        <v>21224</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -6933,10 +6797,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J12" t="n">
+        <v>21224</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -7023,10 +6885,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>11953</t>
-        </is>
+      <c r="J13" t="n">
+        <v>11953</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -7113,10 +6973,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>90034</t>
-        </is>
+      <c r="J14" t="n">
+        <v>90034</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -7203,10 +7061,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>44023</t>
-        </is>
+      <c r="J15" t="n">
+        <v>44023</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -7293,10 +7149,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>78045</t>
-        </is>
+      <c r="J16" t="n">
+        <v>78045</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -7383,10 +7237,8 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>85013</t>
-        </is>
+      <c r="J17" t="n">
+        <v>85013</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -7473,10 +7325,8 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>37110</t>
-        </is>
+      <c r="J18" t="n">
+        <v>37110</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -7563,10 +7413,8 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>53207</t>
-        </is>
+      <c r="J19" t="n">
+        <v>53207</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -7653,10 +7501,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>48180</t>
-        </is>
+      <c r="J20" t="n">
+        <v>48180</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -7743,10 +7589,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>61109</t>
-        </is>
+      <c r="J21" t="n">
+        <v>61109</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -7833,10 +7677,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>19014</t>
-        </is>
+      <c r="J22" t="n">
+        <v>19014</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -7923,10 +7765,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J23" t="n">
+        <v>95111</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -8013,10 +7853,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>75062</t>
-        </is>
+      <c r="J24" t="n">
+        <v>75062</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -8103,10 +7941,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>12204</t>
-        </is>
+      <c r="J25" t="n">
+        <v>12204</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -8193,10 +8029,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J26" t="n">
+        <v>8846</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -8283,10 +8117,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J27" t="n">
+        <v>8846</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -8373,10 +8205,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J28" t="n">
+        <v>8846</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -8463,10 +8293,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J29" t="n">
+        <v>8846</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -8553,10 +8381,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J30" t="n">
+        <v>8846</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -8643,10 +8469,8 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>70116</t>
-        </is>
+      <c r="J31" t="n">
+        <v>70116</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -8733,10 +8557,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>70611</t>
-        </is>
+      <c r="J32" t="n">
+        <v>70611</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -8823,10 +8645,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>8014</t>
-        </is>
+      <c r="J33" t="n">
+        <v>8014</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -8913,10 +8733,8 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>99501</t>
-        </is>
+      <c r="J34" t="n">
+        <v>99501</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -9003,10 +8821,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>45011</t>
-        </is>
+      <c r="J35" t="n">
+        <v>45011</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -9093,10 +8909,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>44805</t>
-        </is>
+      <c r="J36" t="n">
+        <v>44805</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -9183,10 +8997,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>60632</t>
-        </is>
+      <c r="J37" t="n">
+        <v>60632</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -9273,10 +9085,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J38" t="n">
+        <v>95111</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -9363,10 +9173,8 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J39" t="n">
+        <v>95111</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -9453,10 +9261,8 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J40" t="n">
+        <v>21224</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -9543,10 +9349,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J41" t="n">
+        <v>21224</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -9633,10 +9437,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>11953</t>
-        </is>
+      <c r="J42" t="n">
+        <v>11953</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -9723,10 +9525,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>90034</t>
-        </is>
+      <c r="J43" t="n">
+        <v>90034</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -9813,10 +9613,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>44023</t>
-        </is>
+      <c r="J44" t="n">
+        <v>44023</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -9903,10 +9701,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>78045</t>
-        </is>
+      <c r="J45" t="n">
+        <v>78045</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -9993,10 +9789,8 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>85013</t>
-        </is>
+      <c r="J46" t="n">
+        <v>85013</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -10083,10 +9877,8 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>37110</t>
-        </is>
+      <c r="J47" t="n">
+        <v>37110</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -10173,10 +9965,8 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>53207</t>
-        </is>
+      <c r="J48" t="n">
+        <v>53207</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -10263,10 +10053,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>48180</t>
-        </is>
+      <c r="J49" t="n">
+        <v>48180</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -10353,10 +10141,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>61109</t>
-        </is>
+      <c r="J50" t="n">
+        <v>61109</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -10443,10 +10229,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>19014</t>
-        </is>
+      <c r="J51" t="n">
+        <v>19014</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -10533,10 +10317,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J52" t="n">
+        <v>95111</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -10623,10 +10405,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>75062</t>
-        </is>
+      <c r="J53" t="n">
+        <v>75062</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -10713,10 +10493,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>12204</t>
-        </is>
+      <c r="J54" t="n">
+        <v>12204</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -10803,10 +10581,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J55" t="n">
+        <v>8846</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -10893,10 +10669,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J56" t="n">
+        <v>8846</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -10983,10 +10757,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J57" t="n">
+        <v>8846</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -11073,10 +10845,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J58" t="n">
+        <v>8846</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -11163,10 +10933,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J59" t="n">
+        <v>8846</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -11253,10 +11021,8 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>70116</t>
-        </is>
+      <c r="J60" t="n">
+        <v>70116</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -11343,10 +11109,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>70611</t>
-        </is>
+      <c r="J61" t="n">
+        <v>70611</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -11433,10 +11197,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>8014</t>
-        </is>
+      <c r="J62" t="n">
+        <v>8014</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -11523,10 +11285,8 @@
           <t>AK</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>99501</t>
-        </is>
+      <c r="J63" t="n">
+        <v>99501</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -11613,10 +11373,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>45011</t>
-        </is>
+      <c r="J64" t="n">
+        <v>45011</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -11703,10 +11461,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>44805</t>
-        </is>
+      <c r="J65" t="n">
+        <v>44805</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -11793,10 +11549,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>60632</t>
-        </is>
+      <c r="J66" t="n">
+        <v>60632</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -11883,10 +11637,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J67" t="n">
+        <v>95111</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -11973,10 +11725,8 @@
           <t>SD</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J68" t="n">
+        <v>95111</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -12063,10 +11813,8 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J69" t="n">
+        <v>21224</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -12153,10 +11901,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>21224</t>
-        </is>
+      <c r="J70" t="n">
+        <v>21224</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -12243,10 +11989,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>11953</t>
-        </is>
+      <c r="J71" t="n">
+        <v>11953</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -12333,10 +12077,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>90034</t>
-        </is>
+      <c r="J72" t="n">
+        <v>90034</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -12423,10 +12165,8 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>44023</t>
-        </is>
+      <c r="J73" t="n">
+        <v>44023</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -12513,10 +12253,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>78045</t>
-        </is>
+      <c r="J74" t="n">
+        <v>78045</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -12603,10 +12341,8 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>85013</t>
-        </is>
+      <c r="J75" t="n">
+        <v>85013</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -12693,10 +12429,8 @@
           <t>TN</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>37110</t>
-        </is>
+      <c r="J76" t="n">
+        <v>37110</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -12783,10 +12517,8 @@
           <t>WI</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>53207</t>
-        </is>
+      <c r="J77" t="n">
+        <v>53207</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -12873,10 +12605,8 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>48180</t>
-        </is>
+      <c r="J78" t="n">
+        <v>48180</v>
       </c>
       <c r="K78" t="inlineStr">
         <is>
@@ -12963,10 +12693,8 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>61109</t>
-        </is>
+      <c r="J79" t="n">
+        <v>61109</v>
       </c>
       <c r="K79" t="inlineStr">
         <is>
@@ -13053,10 +12781,8 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>19014</t>
-        </is>
+      <c r="J80" t="n">
+        <v>19014</v>
       </c>
       <c r="K80" t="inlineStr">
         <is>
@@ -13143,10 +12869,8 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>95111</t>
-        </is>
+      <c r="J81" t="n">
+        <v>95111</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -13233,10 +12957,8 @@
           <t>TX</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>75062</t>
-        </is>
+      <c r="J82" t="n">
+        <v>75062</v>
       </c>
       <c r="K82" t="inlineStr">
         <is>
@@ -13323,10 +13045,8 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>12204</t>
-        </is>
+      <c r="J83" t="n">
+        <v>12204</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -13413,10 +13133,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J84" t="n">
+        <v>8846</v>
       </c>
       <c r="K84" t="inlineStr">
         <is>
@@ -13503,10 +13221,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J85" t="n">
+        <v>8846</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -13593,10 +13309,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J86" t="n">
+        <v>8846</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -13683,10 +13397,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J87" t="n">
+        <v>8846</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -13773,10 +13485,8 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>8846</t>
-        </is>
+      <c r="J88" t="n">
+        <v>8846</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>

</xml_diff>